<commit_message>
Highlight 920C advantage groups in workbook and README
</commit_message>
<xml_diff>
--- a/experiments/openwiki-optimizer-920c-2026-09/a-baseline-advantage-2026-09-28.xlsx
+++ b/experiments/openwiki-optimizer-920c-2026-09/a-baseline-advantage-2026-09-28.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A组对照" sheetId="1" r:id="Rf37a2cf19b134b02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="组别区别" sheetId="2" r:id="R4319de64a8ec4330"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与限制" sheetId="3" r:id="Rc677b33344eb4556"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A组对照" sheetId="1" r:id="Rcf015cc71b4a4e45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="组别区别" sheetId="2" r:id="R96f17661b484450a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与限制" sheetId="3" r:id="R310c76b639f24a09"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -48,6 +48,12 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17365D"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -90,7 +96,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -118,6 +124,10 @@
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -418,125 +428,125 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="11" t="str">
+      <x:c r="A3" s="25" t="str">
         <x:v>gf_vect_mul</x:v>
       </x:c>
-      <x:c r="B3" s="11" t="str">
+      <x:c r="B3" s="25" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C3" s="11" t="n">
+      <x:c r="C3" s="25" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D3" s="12" t="n">
+      <x:c r="D3" s="26" t="n">
         <x:v>26.78</x:v>
       </x:c>
-      <x:c r="E3" s="12" t="n">
+      <x:c r="E3" s="26" t="n">
         <x:v>6.29</x:v>
       </x:c>
-      <x:c r="F3" s="13" t="n">
+      <x:c r="F3" s="27" t="n">
         <x:v>11652755</x:v>
       </x:c>
-      <x:c r="G3" s="12" t="n">
+      <x:c r="G3" s="26" t="n">
         <x:v>-52.61</x:v>
       </x:c>
-      <x:c r="H3" s="13" t="n">
+      <x:c r="H3" s="27" t="n">
         <x:v>312851</x:v>
       </x:c>
-      <x:c r="I3" s="12" t="n">
+      <x:c r="I3" s="26" t="n">
         <x:v>-28.55</x:v>
       </x:c>
-      <x:c r="J3" s="14" t="n">
+      <x:c r="J3" s="28" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="K3" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L3" s="11" t="str">
+      <x:c r="K3" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L3" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M3" s="11" t="str">
+      <x:c r="M3" s="25" t="str">
         <x:v>性能；总Token；非缓存Token</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="11" t="str">
+      <x:c r="A4" s="25" t="str">
         <x:v>gf_vect_mul</x:v>
       </x:c>
-      <x:c r="B4" s="11" t="str">
+      <x:c r="B4" s="25" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C4" s="11" t="n">
+      <x:c r="C4" s="25" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D4" s="12" t="n">
+      <x:c r="D4" s="26" t="n">
         <x:v>18.31</x:v>
       </x:c>
-      <x:c r="E4" s="12" t="n">
+      <x:c r="E4" s="26" t="n">
         <x:v>-2.19</x:v>
       </x:c>
-      <x:c r="F4" s="13" t="n">
+      <x:c r="F4" s="27" t="n">
         <x:v>9608261</x:v>
       </x:c>
-      <x:c r="G4" s="12" t="n">
+      <x:c r="G4" s="26" t="n">
         <x:v>-60.92</x:v>
       </x:c>
-      <x:c r="H4" s="13" t="n">
+      <x:c r="H4" s="27" t="n">
         <x:v>273605</x:v>
       </x:c>
-      <x:c r="I4" s="12" t="n">
+      <x:c r="I4" s="26" t="n">
         <x:v>-37.51</x:v>
       </x:c>
-      <x:c r="J4" s="14" t="n">
+      <x:c r="J4" s="28" t="n">
         <x:v>35.9</x:v>
       </x:c>
-      <x:c r="K4" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L4" s="11" t="str">
+      <x:c r="K4" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L4" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M4" s="11" t="str">
+      <x:c r="M4" s="25" t="str">
         <x:v>总Token；非缓存Token</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
-      <x:c r="A5" s="11" t="str">
+      <x:c r="A5" s="25" t="str">
         <x:v>gf_vect_mul</x:v>
       </x:c>
-      <x:c r="B5" s="11" t="str">
+      <x:c r="B5" s="25" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="C5" s="11" t="n">
+      <x:c r="C5" s="25" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D5" s="12" t="n">
+      <x:c r="D5" s="26" t="n">
         <x:v>26.28</x:v>
       </x:c>
-      <x:c r="E5" s="12" t="n">
+      <x:c r="E5" s="26" t="n">
         <x:v>5.78</x:v>
       </x:c>
-      <x:c r="F5" s="13" t="n">
+      <x:c r="F5" s="27" t="n">
         <x:v>13291915</x:v>
       </x:c>
-      <x:c r="G5" s="12" t="n">
+      <x:c r="G5" s="26" t="n">
         <x:v>-45.94</x:v>
       </x:c>
-      <x:c r="H5" s="13" t="n">
+      <x:c r="H5" s="27" t="n">
         <x:v>444715</x:v>
       </x:c>
-      <x:c r="I5" s="12" t="n">
+      <x:c r="I5" s="26" t="n">
         <x:v>1.56</x:v>
       </x:c>
-      <x:c r="J5" s="14" t="n">
+      <x:c r="J5" s="28" t="n">
         <x:v>45.7</x:v>
       </x:c>
-      <x:c r="K5" s="14" t="n">
+      <x:c r="K5" s="28" t="n">
         <x:v>2.5</x:v>
       </x:c>
-      <x:c r="L5" s="11" t="str">
+      <x:c r="L5" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M5" s="11" t="str">
+      <x:c r="M5" s="25" t="str">
         <x:v>性能；总Token</x:v>
       </x:c>
     </x:row>
@@ -582,125 +592,125 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
-      <x:c r="A7" s="11" t="str">
+      <x:c r="A7" s="25" t="str">
         <x:v>crc32_ieee</x:v>
       </x:c>
-      <x:c r="B7" s="11" t="str">
+      <x:c r="B7" s="25" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C7" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D7" s="12" t="n">
+      <x:c r="C7" s="25" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D7" s="26" t="n">
         <x:v>49.14</x:v>
       </x:c>
-      <x:c r="E7" s="12" t="n">
+      <x:c r="E7" s="26" t="n">
         <x:v>13.57</x:v>
       </x:c>
-      <x:c r="F7" s="13" t="n">
+      <x:c r="F7" s="27" t="n">
         <x:v>72068320</x:v>
       </x:c>
-      <x:c r="G7" s="12" t="n">
+      <x:c r="G7" s="26" t="n">
         <x:v>-2.84</x:v>
       </x:c>
-      <x:c r="H7" s="13" t="n">
+      <x:c r="H7" s="27" t="n">
         <x:v>886744</x:v>
       </x:c>
-      <x:c r="I7" s="12" t="n">
+      <x:c r="I7" s="26" t="n">
         <x:v>31.75</x:v>
       </x:c>
-      <x:c r="J7" s="14" t="n">
+      <x:c r="J7" s="28" t="n">
         <x:v>119.4</x:v>
       </x:c>
-      <x:c r="K7" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L7" s="11" t="str">
+      <x:c r="K7" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L7" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M7" s="11" t="str">
+      <x:c r="M7" s="25" t="str">
         <x:v>性能；总Token</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
-      <x:c r="A8" s="11" t="str">
+      <x:c r="A8" s="25" t="str">
         <x:v>crc32_ieee</x:v>
       </x:c>
-      <x:c r="B8" s="11" t="str">
+      <x:c r="B8" s="25" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C8" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D8" s="12" t="n">
+      <x:c r="C8" s="25" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D8" s="26" t="n">
         <x:v>28.72</x:v>
       </x:c>
-      <x:c r="E8" s="12" t="n">
+      <x:c r="E8" s="26" t="n">
         <x:v>-6.84</x:v>
       </x:c>
-      <x:c r="F8" s="13" t="n">
+      <x:c r="F8" s="27" t="n">
         <x:v>53206012</x:v>
       </x:c>
-      <x:c r="G8" s="12" t="n">
+      <x:c r="G8" s="26" t="n">
         <x:v>-28.27</x:v>
       </x:c>
-      <x:c r="H8" s="13" t="n">
+      <x:c r="H8" s="27" t="n">
         <x:v>764022</x:v>
       </x:c>
-      <x:c r="I8" s="12" t="n">
+      <x:c r="I8" s="26" t="n">
         <x:v>13.52</x:v>
       </x:c>
-      <x:c r="J8" s="14" t="n">
+      <x:c r="J8" s="28" t="n">
         <x:v>85.6</x:v>
       </x:c>
-      <x:c r="K8" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L8" s="11" t="str">
+      <x:c r="K8" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L8" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M8" s="11" t="str">
+      <x:c r="M8" s="25" t="str">
         <x:v>总Token</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="11" t="str">
+      <x:c r="A9" s="25" t="str">
         <x:v>crc32_ieee</x:v>
       </x:c>
-      <x:c r="B9" s="11" t="str">
+      <x:c r="B9" s="25" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="C9" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D9" s="12" t="n">
+      <x:c r="C9" s="25" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D9" s="26" t="n">
         <x:v>39.12</x:v>
       </x:c>
-      <x:c r="E9" s="12" t="n">
+      <x:c r="E9" s="26" t="n">
         <x:v>3.55</x:v>
       </x:c>
-      <x:c r="F9" s="13" t="n">
+      <x:c r="F9" s="27" t="n">
         <x:v>32444276</x:v>
       </x:c>
-      <x:c r="G9" s="12" t="n">
+      <x:c r="G9" s="26" t="n">
         <x:v>-56.26</x:v>
       </x:c>
-      <x:c r="H9" s="13" t="n">
+      <x:c r="H9" s="27" t="n">
         <x:v>535476</x:v>
       </x:c>
-      <x:c r="I9" s="12" t="n">
+      <x:c r="I9" s="26" t="n">
         <x:v>-20.44</x:v>
       </x:c>
-      <x:c r="J9" s="14" t="n">
+      <x:c r="J9" s="28" t="n">
         <x:v>90.6</x:v>
       </x:c>
-      <x:c r="K9" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L9" s="11" t="str">
+      <x:c r="K9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L9" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M9" s="11" t="str">
+      <x:c r="M9" s="25" t="str">
         <x:v>性能；总Token；非缓存Token</x:v>
       </x:c>
     </x:row>
@@ -746,43 +756,43 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="11" t="str">
+      <x:c r="A11" s="25" t="str">
         <x:v>libm_sin_cos_dp</x:v>
       </x:c>
-      <x:c r="B11" s="11" t="str">
+      <x:c r="B11" s="25" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C11" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D11" s="12" t="n">
+      <x:c r="C11" s="25" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D11" s="26" t="n">
         <x:v>3.63</x:v>
       </x:c>
-      <x:c r="E11" s="12" t="n">
+      <x:c r="E11" s="26" t="n">
         <x:v>-4.47</x:v>
       </x:c>
-      <x:c r="F11" s="13" t="n">
+      <x:c r="F11" s="27" t="n">
         <x:v>23388870</x:v>
       </x:c>
-      <x:c r="G11" s="12" t="n">
+      <x:c r="G11" s="26" t="n">
         <x:v>9.76</x:v>
       </x:c>
-      <x:c r="H11" s="13" t="n">
+      <x:c r="H11" s="27" t="n">
         <x:v>403229</x:v>
       </x:c>
-      <x:c r="I11" s="12" t="n">
+      <x:c r="I11" s="26" t="n">
         <x:v>-6.64</x:v>
       </x:c>
-      <x:c r="J11" s="14" t="n">
+      <x:c r="J11" s="28" t="n">
         <x:v>47.1</x:v>
       </x:c>
-      <x:c r="K11" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L11" s="11" t="str">
+      <x:c r="K11" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L11" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M11" s="11" t="str">
+      <x:c r="M11" s="25" t="str">
         <x:v>非缓存Token</x:v>
       </x:c>
     </x:row>
@@ -910,125 +920,125 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="11" t="str">
+      <x:c r="A15" s="25" t="str">
         <x:v>dftbench_double</x:v>
       </x:c>
-      <x:c r="B15" s="11" t="str">
+      <x:c r="B15" s="25" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C15" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D15" s="12" t="n">
+      <x:c r="C15" s="25" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D15" s="26" t="n">
         <x:v>22.3</x:v>
       </x:c>
-      <x:c r="E15" s="12" t="n">
+      <x:c r="E15" s="26" t="n">
         <x:v>-0.75</x:v>
       </x:c>
-      <x:c r="F15" s="13" t="n">
+      <x:c r="F15" s="27" t="n">
         <x:v>30858303</x:v>
       </x:c>
-      <x:c r="G15" s="12" t="n">
+      <x:c r="G15" s="26" t="n">
         <x:v>-40.63</x:v>
       </x:c>
-      <x:c r="H15" s="13" t="n">
+      <x:c r="H15" s="27" t="n">
         <x:v>467014</x:v>
       </x:c>
-      <x:c r="I15" s="12" t="n">
+      <x:c r="I15" s="26" t="n">
         <x:v>-7.57</x:v>
       </x:c>
-      <x:c r="J15" s="14" t="n">
+      <x:c r="J15" s="28" t="n">
         <x:v>60.1</x:v>
       </x:c>
-      <x:c r="K15" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L15" s="11" t="str">
+      <x:c r="K15" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L15" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M15" s="11" t="str">
+      <x:c r="M15" s="25" t="str">
         <x:v>总Token；非缓存Token</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="11" t="str">
+      <x:c r="A16" s="25" t="str">
         <x:v>dftbench_double</x:v>
       </x:c>
-      <x:c r="B16" s="11" t="str">
+      <x:c r="B16" s="25" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C16" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D16" s="12" t="n">
+      <x:c r="C16" s="25" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D16" s="26" t="n">
         <x:v>23.8</x:v>
       </x:c>
-      <x:c r="E16" s="12" t="n">
+      <x:c r="E16" s="26" t="n">
         <x:v>0.76</x:v>
       </x:c>
-      <x:c r="F16" s="13" t="n">
+      <x:c r="F16" s="27" t="n">
         <x:v>42683881</x:v>
       </x:c>
-      <x:c r="G16" s="12" t="n">
+      <x:c r="G16" s="26" t="n">
         <x:v>-17.87</x:v>
       </x:c>
-      <x:c r="H16" s="13" t="n">
+      <x:c r="H16" s="27" t="n">
         <x:v>444764</x:v>
       </x:c>
-      <x:c r="I16" s="12" t="n">
+      <x:c r="I16" s="26" t="n">
         <x:v>-11.97</x:v>
       </x:c>
-      <x:c r="J16" s="14" t="n">
+      <x:c r="J16" s="28" t="n">
         <x:v>74.3</x:v>
       </x:c>
-      <x:c r="K16" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L16" s="11" t="str">
+      <x:c r="K16" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L16" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M16" s="11" t="str">
+      <x:c r="M16" s="25" t="str">
         <x:v>性能；总Token；非缓存Token</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="11" t="str">
+      <x:c r="A17" s="25" t="str">
         <x:v>dftbench_double</x:v>
       </x:c>
-      <x:c r="B17" s="11" t="str">
+      <x:c r="B17" s="25" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="C17" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D17" s="12" t="n">
+      <x:c r="C17" s="25" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D17" s="26" t="n">
         <x:v>31.29</x:v>
       </x:c>
-      <x:c r="E17" s="12" t="n">
+      <x:c r="E17" s="26" t="n">
         <x:v>8.25</x:v>
       </x:c>
-      <x:c r="F17" s="13" t="n">
+      <x:c r="F17" s="27" t="n">
         <x:v>30752047</x:v>
       </x:c>
-      <x:c r="G17" s="12" t="n">
+      <x:c r="G17" s="26" t="n">
         <x:v>-40.83</x:v>
       </x:c>
-      <x:c r="H17" s="13" t="n">
+      <x:c r="H17" s="27" t="n">
         <x:v>653685</x:v>
       </x:c>
-      <x:c r="I17" s="12" t="n">
+      <x:c r="I17" s="26" t="n">
         <x:v>29.38</x:v>
       </x:c>
-      <x:c r="J17" s="14" t="n">
+      <x:c r="J17" s="28" t="n">
         <x:v>82.8</x:v>
       </x:c>
-      <x:c r="K17" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L17" s="11" t="str">
+      <x:c r="K17" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L17" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M17" s="11" t="str">
+      <x:c r="M17" s="25" t="str">
         <x:v>性能；总Token</x:v>
       </x:c>
     </x:row>
@@ -1115,84 +1125,84 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
-      <x:c r="A20" s="11" t="str">
+      <x:c r="A20" s="25" t="str">
         <x:v>tlfloat_quad_arithmetic</x:v>
       </x:c>
-      <x:c r="B20" s="11" t="str">
+      <x:c r="B20" s="25" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C20" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D20" s="12" t="n">
+      <x:c r="C20" s="25" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D20" s="26" t="n">
         <x:v>15.78</x:v>
       </x:c>
-      <x:c r="E20" s="12" t="n">
+      <x:c r="E20" s="26" t="n">
         <x:v>9.72</x:v>
       </x:c>
-      <x:c r="F20" s="13" t="n">
+      <x:c r="F20" s="27" t="n">
         <x:v>28139344</x:v>
       </x:c>
-      <x:c r="G20" s="12" t="n">
+      <x:c r="G20" s="26" t="n">
         <x:v>33.55</x:v>
       </x:c>
-      <x:c r="H20" s="13" t="n">
+      <x:c r="H20" s="27" t="n">
         <x:v>487120</x:v>
       </x:c>
-      <x:c r="I20" s="12" t="n">
+      <x:c r="I20" s="26" t="n">
         <x:v>10.88</x:v>
       </x:c>
-      <x:c r="J20" s="14" t="n">
+      <x:c r="J20" s="28" t="n">
         <x:v>80.2</x:v>
       </x:c>
-      <x:c r="K20" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L20" s="11" t="str">
+      <x:c r="K20" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L20" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M20" s="11" t="str">
+      <x:c r="M20" s="25" t="str">
         <x:v>性能</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
-      <x:c r="A21" s="11" t="str">
+      <x:c r="A21" s="25" t="str">
         <x:v>tlfloat_quad_arithmetic</x:v>
       </x:c>
-      <x:c r="B21" s="11" t="str">
+      <x:c r="B21" s="25" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="C21" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D21" s="12" t="n">
+      <x:c r="C21" s="25" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D21" s="26" t="n">
         <x:v>3.67</x:v>
       </x:c>
-      <x:c r="E21" s="12" t="n">
+      <x:c r="E21" s="26" t="n">
         <x:v>-2.39</x:v>
       </x:c>
-      <x:c r="F21" s="13" t="n">
+      <x:c r="F21" s="27" t="n">
         <x:v>35644212</x:v>
       </x:c>
-      <x:c r="G21" s="12" t="n">
+      <x:c r="G21" s="26" t="n">
         <x:v>69.17</x:v>
       </x:c>
-      <x:c r="H21" s="13" t="n">
+      <x:c r="H21" s="27" t="n">
         <x:v>430132</x:v>
       </x:c>
-      <x:c r="I21" s="12" t="n">
+      <x:c r="I21" s="26" t="n">
         <x:v>-2.1</x:v>
       </x:c>
-      <x:c r="J21" s="14" t="n">
+      <x:c r="J21" s="28" t="n">
         <x:v>89.8</x:v>
       </x:c>
-      <x:c r="K21" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L21" s="11" t="str">
+      <x:c r="K21" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L21" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M21" s="11" t="str">
+      <x:c r="M21" s="25" t="str">
         <x:v>非缓存Token</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Frame each operator group without workbook fills
</commit_message>
<xml_diff>
--- a/experiments/openwiki-optimizer-920c-2026-09/a-baseline-advantage-2026-09-28.xlsx
+++ b/experiments/openwiki-optimizer-920c-2026-09/a-baseline-advantage-2026-09-28.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A组对照" sheetId="1" r:id="Rcf015cc71b4a4e45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="组别区别" sheetId="2" r:id="R96f17661b484450a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与限制" sheetId="3" r:id="R310c76b639f24a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A组对照" sheetId="1" r:id="Ra78bed7b4ae24083"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="组别区别" sheetId="2" r:id="R2619c228e24f459e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与限制" sheetId="3" r:id="R6b63534008bc4d1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -54,6 +54,18 @@
       <x:b/>
       <x:sz val="10"/>
       <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF222222"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -90,13 +102,65 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="9">
     <x:border/>
+    <x:border>
+      <x:left style="thick">
+        <x:color rgb="FF333333"/>
+      </x:left>
+      <x:top style="thick">
+        <x:color rgb="FF333333"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thick">
+        <x:color rgb="FF333333"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thick">
+        <x:color rgb="FF333333"/>
+      </x:right>
+      <x:top style="thick">
+        <x:color rgb="FF333333"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thick">
+        <x:color rgb="FF333333"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thick">
+        <x:color rgb="FF333333"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thick">
+        <x:color rgb="FF333333"/>
+      </x:left>
+      <x:bottom style="thick">
+        <x:color rgb="FF333333"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thick">
+        <x:color rgb="FF333333"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thick">
+        <x:color rgb="FF333333"/>
+      </x:right>
+      <x:bottom style="thick">
+        <x:color rgb="FF333333"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="29">
+  <x:cellXfs count="74">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -128,6 +192,53 @@
     <x:xf numFmtId="200" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="1" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="1" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="1" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="1" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0"/>
+    <x:xf numFmtId="200" fontId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0"/>
+    <x:xf numFmtId="201" fontId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0"/>
+    <x:xf numFmtId="202" fontId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0"/>
+    <x:xf numFmtId="200" fontId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0"/>
+    <x:xf numFmtId="201" fontId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0"/>
+    <x:xf numFmtId="202" fontId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="1" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="1" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="1" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -346,904 +457,919 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="29" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="42" t="str">
         <x:v>算子</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" s="42" t="str">
         <x:v>组别</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="str">
+      <x:c r="C1" s="42" t="str">
         <x:v>可比轮次</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
+      <x:c r="D1" s="42" t="str">
         <x:v>得分(%)</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="str">
+      <x:c r="E1" s="42" t="str">
         <x:v>diff(pp)</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="str">
+      <x:c r="F1" s="42" t="str">
         <x:v>总Token</x:v>
       </x:c>
-      <x:c r="G1" s="3" t="str">
+      <x:c r="G1" s="42" t="str">
         <x:v>总Token较A(%)</x:v>
       </x:c>
-      <x:c r="H1" s="3" t="str">
+      <x:c r="H1" s="42" t="str">
         <x:v>非缓存Token</x:v>
       </x:c>
-      <x:c r="I1" s="3" t="str">
+      <x:c r="I1" s="42" t="str">
         <x:v>非缓存Token较A(%)</x:v>
       </x:c>
-      <x:c r="J1" s="3" t="str">
+      <x:c r="J1" s="42" t="str">
         <x:v>耗时中位数(分钟)</x:v>
       </x:c>
-      <x:c r="K1" s="3" t="str">
+      <x:c r="K1" s="42" t="str">
         <x:v>平均迭代轮数</x:v>
       </x:c>
-      <x:c r="L1" s="3" t="str">
+      <x:c r="L1" s="42" t="str">
         <x:v>优势组</x:v>
       </x:c>
-      <x:c r="M1" s="3" t="str">
+      <x:c r="M1" s="42" t="str">
         <x:v>优势依据</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="7" t="str">
+      <x:c r="A2" s="44" t="str">
         <x:v>gf_vect_mul</x:v>
       </x:c>
-      <x:c r="B2" s="7" t="str">
+      <x:c r="B2" s="45" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="C2" s="7" t="n">
+      <x:c r="C2" s="45" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D2" s="8" t="n">
+      <x:c r="D2" s="46" t="n">
         <x:v>20.5</x:v>
       </x:c>
-      <x:c r="E2" s="8" t="n">
+      <x:c r="E2" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F2" s="9" t="n">
+      <x:c r="F2" s="47" t="n">
         <x:v>24589065</x:v>
       </x:c>
-      <x:c r="G2" s="8" t="n">
+      <x:c r="G2" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H2" s="9" t="n">
+      <x:c r="H2" s="47" t="n">
         <x:v>437865</x:v>
       </x:c>
-      <x:c r="I2" s="8" t="n">
+      <x:c r="I2" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J2" s="10" t="n">
+      <x:c r="J2" s="48" t="n">
         <x:v>60.7</x:v>
       </x:c>
-      <x:c r="K2" s="10" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L2" s="7" t="str">
+      <x:c r="K2" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L2" s="45" t="str">
         <x:v>对照</x:v>
       </x:c>
-      <x:c r="M2" s="7" t="str">
+      <x:c r="M2" s="49" t="str">
         <x:v>无</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="25" t="str">
+      <x:c r="A3" s="50" t="str">
         <x:v>gf_vect_mul</x:v>
       </x:c>
-      <x:c r="B3" s="25" t="str">
+      <x:c r="B3" s="51" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C3" s="25" t="n">
+      <x:c r="C3" s="51" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D3" s="26" t="n">
+      <x:c r="D3" s="52" t="n">
         <x:v>26.78</x:v>
       </x:c>
-      <x:c r="E3" s="26" t="n">
+      <x:c r="E3" s="52" t="n">
         <x:v>6.29</x:v>
       </x:c>
-      <x:c r="F3" s="27" t="n">
+      <x:c r="F3" s="53" t="n">
         <x:v>11652755</x:v>
       </x:c>
-      <x:c r="G3" s="26" t="n">
+      <x:c r="G3" s="52" t="n">
         <x:v>-52.61</x:v>
       </x:c>
-      <x:c r="H3" s="27" t="n">
+      <x:c r="H3" s="53" t="n">
         <x:v>312851</x:v>
       </x:c>
-      <x:c r="I3" s="26" t="n">
+      <x:c r="I3" s="52" t="n">
         <x:v>-28.55</x:v>
       </x:c>
-      <x:c r="J3" s="28" t="n">
+      <x:c r="J3" s="54" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="K3" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L3" s="25" t="str">
+      <x:c r="K3" s="54" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L3" s="51" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M3" s="25" t="str">
+      <x:c r="M3" s="55" t="str">
         <x:v>性能；总Token；非缓存Token</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="25" t="str">
+      <x:c r="A4" s="50" t="str">
         <x:v>gf_vect_mul</x:v>
       </x:c>
-      <x:c r="B4" s="25" t="str">
+      <x:c r="B4" s="51" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C4" s="25" t="n">
+      <x:c r="C4" s="51" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D4" s="26" t="n">
+      <x:c r="D4" s="52" t="n">
         <x:v>18.31</x:v>
       </x:c>
-      <x:c r="E4" s="26" t="n">
+      <x:c r="E4" s="52" t="n">
         <x:v>-2.19</x:v>
       </x:c>
-      <x:c r="F4" s="27" t="n">
+      <x:c r="F4" s="53" t="n">
         <x:v>9608261</x:v>
       </x:c>
-      <x:c r="G4" s="26" t="n">
+      <x:c r="G4" s="52" t="n">
         <x:v>-60.92</x:v>
       </x:c>
-      <x:c r="H4" s="27" t="n">
+      <x:c r="H4" s="53" t="n">
         <x:v>273605</x:v>
       </x:c>
-      <x:c r="I4" s="26" t="n">
+      <x:c r="I4" s="52" t="n">
         <x:v>-37.51</x:v>
       </x:c>
-      <x:c r="J4" s="28" t="n">
+      <x:c r="J4" s="54" t="n">
         <x:v>35.9</x:v>
       </x:c>
-      <x:c r="K4" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L4" s="25" t="str">
+      <x:c r="K4" s="54" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L4" s="51" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M4" s="25" t="str">
+      <x:c r="M4" s="55" t="str">
         <x:v>总Token；非缓存Token</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
-      <x:c r="A5" s="25" t="str">
+      <x:c r="A5" s="56" t="str">
         <x:v>gf_vect_mul</x:v>
       </x:c>
-      <x:c r="B5" s="25" t="str">
+      <x:c r="B5" s="57" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="C5" s="25" t="n">
+      <x:c r="C5" s="57" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D5" s="26" t="n">
+      <x:c r="D5" s="58" t="n">
         <x:v>26.28</x:v>
       </x:c>
-      <x:c r="E5" s="26" t="n">
+      <x:c r="E5" s="58" t="n">
         <x:v>5.78</x:v>
       </x:c>
-      <x:c r="F5" s="27" t="n">
+      <x:c r="F5" s="59" t="n">
         <x:v>13291915</x:v>
       </x:c>
-      <x:c r="G5" s="26" t="n">
+      <x:c r="G5" s="58" t="n">
         <x:v>-45.94</x:v>
       </x:c>
-      <x:c r="H5" s="27" t="n">
+      <x:c r="H5" s="59" t="n">
         <x:v>444715</x:v>
       </x:c>
-      <x:c r="I5" s="26" t="n">
+      <x:c r="I5" s="58" t="n">
         <x:v>1.56</x:v>
       </x:c>
-      <x:c r="J5" s="28" t="n">
+      <x:c r="J5" s="60" t="n">
         <x:v>45.7</x:v>
       </x:c>
-      <x:c r="K5" s="28" t="n">
+      <x:c r="K5" s="60" t="n">
         <x:v>2.5</x:v>
       </x:c>
-      <x:c r="L5" s="25" t="str">
+      <x:c r="L5" s="57" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M5" s="25" t="str">
+      <x:c r="M5" s="61" t="str">
         <x:v>性能；总Token</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="7" t="str">
+      <x:c r="A6" s="44" t="str">
         <x:v>crc32_ieee</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="str">
+      <x:c r="B6" s="45" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D6" s="8" t="n">
+      <x:c r="C6" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D6" s="46" t="n">
         <x:v>35.57</x:v>
       </x:c>
-      <x:c r="E6" s="8" t="n">
+      <x:c r="E6" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F6" s="9" t="n">
+      <x:c r="F6" s="47" t="n">
         <x:v>74177453</x:v>
       </x:c>
-      <x:c r="G6" s="8" t="n">
+      <x:c r="G6" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H6" s="9" t="n">
+      <x:c r="H6" s="47" t="n">
         <x:v>673029</x:v>
       </x:c>
-      <x:c r="I6" s="8" t="n">
+      <x:c r="I6" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J6" s="10" t="n">
+      <x:c r="J6" s="48" t="n">
         <x:v>89.3</x:v>
       </x:c>
-      <x:c r="K6" s="10" t="n">
+      <x:c r="K6" s="48" t="n">
         <x:v>2.7</x:v>
       </x:c>
-      <x:c r="L6" s="7" t="str">
+      <x:c r="L6" s="45" t="str">
         <x:v>对照</x:v>
       </x:c>
-      <x:c r="M6" s="7" t="str">
+      <x:c r="M6" s="49" t="str">
         <x:v>无</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
-      <x:c r="A7" s="25" t="str">
+      <x:c r="A7" s="50" t="str">
         <x:v>crc32_ieee</x:v>
       </x:c>
-      <x:c r="B7" s="25" t="str">
+      <x:c r="B7" s="51" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C7" s="25" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D7" s="26" t="n">
+      <x:c r="C7" s="51" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D7" s="52" t="n">
         <x:v>49.14</x:v>
       </x:c>
-      <x:c r="E7" s="26" t="n">
+      <x:c r="E7" s="52" t="n">
         <x:v>13.57</x:v>
       </x:c>
-      <x:c r="F7" s="27" t="n">
+      <x:c r="F7" s="53" t="n">
         <x:v>72068320</x:v>
       </x:c>
-      <x:c r="G7" s="26" t="n">
+      <x:c r="G7" s="52" t="n">
         <x:v>-2.84</x:v>
       </x:c>
-      <x:c r="H7" s="27" t="n">
+      <x:c r="H7" s="53" t="n">
         <x:v>886744</x:v>
       </x:c>
-      <x:c r="I7" s="26" t="n">
+      <x:c r="I7" s="52" t="n">
         <x:v>31.75</x:v>
       </x:c>
-      <x:c r="J7" s="28" t="n">
+      <x:c r="J7" s="54" t="n">
         <x:v>119.4</x:v>
       </x:c>
-      <x:c r="K7" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L7" s="25" t="str">
+      <x:c r="K7" s="54" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L7" s="51" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M7" s="25" t="str">
+      <x:c r="M7" s="55" t="str">
         <x:v>性能；总Token</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
-      <x:c r="A8" s="25" t="str">
+      <x:c r="A8" s="50" t="str">
         <x:v>crc32_ieee</x:v>
       </x:c>
-      <x:c r="B8" s="25" t="str">
+      <x:c r="B8" s="51" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C8" s="25" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D8" s="26" t="n">
+      <x:c r="C8" s="51" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D8" s="52" t="n">
         <x:v>28.72</x:v>
       </x:c>
-      <x:c r="E8" s="26" t="n">
+      <x:c r="E8" s="52" t="n">
         <x:v>-6.84</x:v>
       </x:c>
-      <x:c r="F8" s="27" t="n">
+      <x:c r="F8" s="53" t="n">
         <x:v>53206012</x:v>
       </x:c>
-      <x:c r="G8" s="26" t="n">
+      <x:c r="G8" s="52" t="n">
         <x:v>-28.27</x:v>
       </x:c>
-      <x:c r="H8" s="27" t="n">
+      <x:c r="H8" s="53" t="n">
         <x:v>764022</x:v>
       </x:c>
-      <x:c r="I8" s="26" t="n">
+      <x:c r="I8" s="52" t="n">
         <x:v>13.52</x:v>
       </x:c>
-      <x:c r="J8" s="28" t="n">
+      <x:c r="J8" s="54" t="n">
         <x:v>85.6</x:v>
       </x:c>
-      <x:c r="K8" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L8" s="25" t="str">
+      <x:c r="K8" s="54" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L8" s="51" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M8" s="25" t="str">
+      <x:c r="M8" s="55" t="str">
         <x:v>总Token</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="25" t="str">
+      <x:c r="A9" s="56" t="str">
         <x:v>crc32_ieee</x:v>
       </x:c>
-      <x:c r="B9" s="25" t="str">
+      <x:c r="B9" s="57" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="C9" s="25" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D9" s="26" t="n">
+      <x:c r="C9" s="57" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D9" s="58" t="n">
         <x:v>39.12</x:v>
       </x:c>
-      <x:c r="E9" s="26" t="n">
+      <x:c r="E9" s="58" t="n">
         <x:v>3.55</x:v>
       </x:c>
-      <x:c r="F9" s="27" t="n">
+      <x:c r="F9" s="59" t="n">
         <x:v>32444276</x:v>
       </x:c>
-      <x:c r="G9" s="26" t="n">
+      <x:c r="G9" s="58" t="n">
         <x:v>-56.26</x:v>
       </x:c>
-      <x:c r="H9" s="27" t="n">
+      <x:c r="H9" s="59" t="n">
         <x:v>535476</x:v>
       </x:c>
-      <x:c r="I9" s="26" t="n">
+      <x:c r="I9" s="58" t="n">
         <x:v>-20.44</x:v>
       </x:c>
-      <x:c r="J9" s="28" t="n">
+      <x:c r="J9" s="60" t="n">
         <x:v>90.6</x:v>
       </x:c>
-      <x:c r="K9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L9" s="25" t="str">
+      <x:c r="K9" s="60" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L9" s="57" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M9" s="25" t="str">
+      <x:c r="M9" s="61" t="str">
         <x:v>性能；总Token；非缓存Token</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="7" t="str">
+      <x:c r="A10" s="44" t="str">
         <x:v>libm_sin_cos_dp</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="str">
+      <x:c r="B10" s="45" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="C10" s="7" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D10" s="8" t="n">
+      <x:c r="C10" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D10" s="46" t="n">
         <x:v>8.1</x:v>
       </x:c>
-      <x:c r="E10" s="8" t="n">
+      <x:c r="E10" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F10" s="9" t="n">
+      <x:c r="F10" s="47" t="n">
         <x:v>21308341</x:v>
       </x:c>
-      <x:c r="G10" s="8" t="n">
+      <x:c r="G10" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H10" s="9" t="n">
+      <x:c r="H10" s="47" t="n">
         <x:v>431885</x:v>
       </x:c>
-      <x:c r="I10" s="8" t="n">
+      <x:c r="I10" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J10" s="10" t="n">
+      <x:c r="J10" s="48" t="n">
         <x:v>43.9</x:v>
       </x:c>
-      <x:c r="K10" s="10" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L10" s="7" t="str">
+      <x:c r="K10" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L10" s="45" t="str">
         <x:v>对照</x:v>
       </x:c>
-      <x:c r="M10" s="7" t="str">
+      <x:c r="M10" s="49" t="str">
         <x:v>无</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="25" t="str">
+      <x:c r="A11" s="50" t="str">
         <x:v>libm_sin_cos_dp</x:v>
       </x:c>
-      <x:c r="B11" s="25" t="str">
+      <x:c r="B11" s="51" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C11" s="25" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D11" s="26" t="n">
+      <x:c r="C11" s="51" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D11" s="52" t="n">
         <x:v>3.63</x:v>
       </x:c>
-      <x:c r="E11" s="26" t="n">
+      <x:c r="E11" s="52" t="n">
         <x:v>-4.47</x:v>
       </x:c>
-      <x:c r="F11" s="27" t="n">
+      <x:c r="F11" s="53" t="n">
         <x:v>23388870</x:v>
       </x:c>
-      <x:c r="G11" s="26" t="n">
+      <x:c r="G11" s="52" t="n">
         <x:v>9.76</x:v>
       </x:c>
-      <x:c r="H11" s="27" t="n">
+      <x:c r="H11" s="53" t="n">
         <x:v>403229</x:v>
       </x:c>
-      <x:c r="I11" s="26" t="n">
+      <x:c r="I11" s="52" t="n">
         <x:v>-6.64</x:v>
       </x:c>
-      <x:c r="J11" s="28" t="n">
+      <x:c r="J11" s="54" t="n">
         <x:v>47.1</x:v>
       </x:c>
-      <x:c r="K11" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L11" s="25" t="str">
+      <x:c r="K11" s="54" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L11" s="51" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M11" s="25" t="str">
+      <x:c r="M11" s="55" t="str">
         <x:v>非缓存Token</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="15" t="str">
+      <x:c r="A12" s="62" t="str">
         <x:v>libm_sin_cos_dp</x:v>
       </x:c>
-      <x:c r="B12" s="15" t="str">
+      <x:c r="B12" s="63" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C12" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D12" s="16" t="n">
+      <x:c r="C12" s="63" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D12" s="64" t="n">
         <x:v>4.98</x:v>
       </x:c>
-      <x:c r="E12" s="16" t="n">
+      <x:c r="E12" s="64" t="n">
         <x:v>-3.13</x:v>
       </x:c>
-      <x:c r="F12" s="17" t="n">
+      <x:c r="F12" s="65" t="n">
         <x:v>23787057</x:v>
       </x:c>
-      <x:c r="G12" s="16" t="n">
+      <x:c r="G12" s="64" t="n">
         <x:v>11.63</x:v>
       </x:c>
-      <x:c r="H12" s="17" t="n">
+      <x:c r="H12" s="65" t="n">
         <x:v>447985</x:v>
       </x:c>
-      <x:c r="I12" s="16" t="n">
+      <x:c r="I12" s="64" t="n">
         <x:v>3.73</x:v>
       </x:c>
-      <x:c r="J12" s="18" t="n">
+      <x:c r="J12" s="66" t="n">
         <x:v>42.5</x:v>
       </x:c>
-      <x:c r="K12" s="18" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L12" s="15" t="str">
+      <x:c r="K12" s="66" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L12" s="63" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="M12" s="15" t="str">
+      <x:c r="M12" s="67" t="str">
         <x:v>无</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="15" t="str">
+      <x:c r="A13" s="68" t="str">
         <x:v>libm_sin_cos_dp</x:v>
       </x:c>
-      <x:c r="B13" s="15" t="str">
+      <x:c r="B13" s="69" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="C13" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D13" s="16" t="n">
+      <x:c r="C13" s="69" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D13" s="70" t="n">
         <x:v>2.36</x:v>
       </x:c>
-      <x:c r="E13" s="16" t="n">
+      <x:c r="E13" s="70" t="n">
         <x:v>-5.74</x:v>
       </x:c>
-      <x:c r="F13" s="17" t="n">
+      <x:c r="F13" s="71" t="n">
         <x:v>38839494</x:v>
       </x:c>
-      <x:c r="G13" s="16" t="n">
+      <x:c r="G13" s="70" t="n">
         <x:v>82.27</x:v>
       </x:c>
-      <x:c r="H13" s="17" t="n">
+      <x:c r="H13" s="71" t="n">
         <x:v>628022</x:v>
       </x:c>
-      <x:c r="I13" s="16" t="n">
+      <x:c r="I13" s="70" t="n">
         <x:v>45.41</x:v>
       </x:c>
-      <x:c r="J13" s="18" t="n">
+      <x:c r="J13" s="72" t="n">
         <x:v>73.5</x:v>
       </x:c>
-      <x:c r="K13" s="18" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L13" s="15" t="str">
+      <x:c r="K13" s="72" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L13" s="69" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="M13" s="15" t="str">
+      <x:c r="M13" s="73" t="str">
         <x:v>无</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="7" t="str">
+      <x:c r="A14" s="44" t="str">
         <x:v>dftbench_double</x:v>
       </x:c>
-      <x:c r="B14" s="7" t="str">
+      <x:c r="B14" s="45" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="C14" s="7" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D14" s="8" t="n">
+      <x:c r="C14" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D14" s="46" t="n">
         <x:v>23.05</x:v>
       </x:c>
-      <x:c r="E14" s="8" t="n">
+      <x:c r="E14" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F14" s="9" t="n">
+      <x:c r="F14" s="47" t="n">
         <x:v>51972520</x:v>
       </x:c>
-      <x:c r="G14" s="8" t="n">
+      <x:c r="G14" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H14" s="9" t="n">
+      <x:c r="H14" s="47" t="n">
         <x:v>505256</x:v>
       </x:c>
-      <x:c r="I14" s="8" t="n">
+      <x:c r="I14" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J14" s="10" t="n">
+      <x:c r="J14" s="48" t="n">
         <x:v>102.4</x:v>
       </x:c>
-      <x:c r="K14" s="10" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L14" s="7" t="str">
+      <x:c r="K14" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L14" s="45" t="str">
         <x:v>对照</x:v>
       </x:c>
-      <x:c r="M14" s="7" t="str">
+      <x:c r="M14" s="49" t="str">
         <x:v>无</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="25" t="str">
+      <x:c r="A15" s="50" t="str">
         <x:v>dftbench_double</x:v>
       </x:c>
-      <x:c r="B15" s="25" t="str">
+      <x:c r="B15" s="51" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C15" s="25" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D15" s="26" t="n">
+      <x:c r="C15" s="51" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D15" s="52" t="n">
         <x:v>22.3</x:v>
       </x:c>
-      <x:c r="E15" s="26" t="n">
+      <x:c r="E15" s="52" t="n">
         <x:v>-0.75</x:v>
       </x:c>
-      <x:c r="F15" s="27" t="n">
+      <x:c r="F15" s="53" t="n">
         <x:v>30858303</x:v>
       </x:c>
-      <x:c r="G15" s="26" t="n">
+      <x:c r="G15" s="52" t="n">
         <x:v>-40.63</x:v>
       </x:c>
-      <x:c r="H15" s="27" t="n">
+      <x:c r="H15" s="53" t="n">
         <x:v>467014</x:v>
       </x:c>
-      <x:c r="I15" s="26" t="n">
+      <x:c r="I15" s="52" t="n">
         <x:v>-7.57</x:v>
       </x:c>
-      <x:c r="J15" s="28" t="n">
+      <x:c r="J15" s="54" t="n">
         <x:v>60.1</x:v>
       </x:c>
-      <x:c r="K15" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L15" s="25" t="str">
+      <x:c r="K15" s="54" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L15" s="51" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M15" s="25" t="str">
+      <x:c r="M15" s="55" t="str">
         <x:v>总Token；非缓存Token</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="25" t="str">
+      <x:c r="A16" s="50" t="str">
         <x:v>dftbench_double</x:v>
       </x:c>
-      <x:c r="B16" s="25" t="str">
+      <x:c r="B16" s="51" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C16" s="25" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D16" s="26" t="n">
+      <x:c r="C16" s="51" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D16" s="52" t="n">
         <x:v>23.8</x:v>
       </x:c>
-      <x:c r="E16" s="26" t="n">
+      <x:c r="E16" s="52" t="n">
         <x:v>0.76</x:v>
       </x:c>
-      <x:c r="F16" s="27" t="n">
+      <x:c r="F16" s="53" t="n">
         <x:v>42683881</x:v>
       </x:c>
-      <x:c r="G16" s="26" t="n">
+      <x:c r="G16" s="52" t="n">
         <x:v>-17.87</x:v>
       </x:c>
-      <x:c r="H16" s="27" t="n">
+      <x:c r="H16" s="53" t="n">
         <x:v>444764</x:v>
       </x:c>
-      <x:c r="I16" s="26" t="n">
+      <x:c r="I16" s="52" t="n">
         <x:v>-11.97</x:v>
       </x:c>
-      <x:c r="J16" s="28" t="n">
+      <x:c r="J16" s="54" t="n">
         <x:v>74.3</x:v>
       </x:c>
-      <x:c r="K16" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L16" s="25" t="str">
+      <x:c r="K16" s="54" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L16" s="51" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M16" s="25" t="str">
+      <x:c r="M16" s="55" t="str">
         <x:v>性能；总Token；非缓存Token</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="25" t="str">
+      <x:c r="A17" s="56" t="str">
         <x:v>dftbench_double</x:v>
       </x:c>
-      <x:c r="B17" s="25" t="str">
+      <x:c r="B17" s="57" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="C17" s="25" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D17" s="26" t="n">
+      <x:c r="C17" s="57" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D17" s="58" t="n">
         <x:v>31.29</x:v>
       </x:c>
-      <x:c r="E17" s="26" t="n">
+      <x:c r="E17" s="58" t="n">
         <x:v>8.25</x:v>
       </x:c>
-      <x:c r="F17" s="27" t="n">
+      <x:c r="F17" s="59" t="n">
         <x:v>30752047</x:v>
       </x:c>
-      <x:c r="G17" s="26" t="n">
+      <x:c r="G17" s="58" t="n">
         <x:v>-40.83</x:v>
       </x:c>
-      <x:c r="H17" s="27" t="n">
+      <x:c r="H17" s="59" t="n">
         <x:v>653685</x:v>
       </x:c>
-      <x:c r="I17" s="26" t="n">
+      <x:c r="I17" s="58" t="n">
         <x:v>29.38</x:v>
       </x:c>
-      <x:c r="J17" s="28" t="n">
+      <x:c r="J17" s="60" t="n">
         <x:v>82.8</x:v>
       </x:c>
-      <x:c r="K17" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L17" s="25" t="str">
+      <x:c r="K17" s="60" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L17" s="57" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M17" s="25" t="str">
+      <x:c r="M17" s="61" t="str">
         <x:v>性能；总Token</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="7" t="str">
+      <x:c r="A18" s="44" t="str">
         <x:v>tlfloat_quad_arithmetic</x:v>
       </x:c>
-      <x:c r="B18" s="7" t="str">
+      <x:c r="B18" s="45" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="C18" s="7" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D18" s="8" t="n">
+      <x:c r="C18" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D18" s="46" t="n">
         <x:v>6.06</x:v>
       </x:c>
-      <x:c r="E18" s="8" t="n">
+      <x:c r="E18" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F18" s="9" t="n">
+      <x:c r="F18" s="47" t="n">
         <x:v>21070214</x:v>
       </x:c>
-      <x:c r="G18" s="8" t="n">
+      <x:c r="G18" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H18" s="9" t="n">
+      <x:c r="H18" s="47" t="n">
         <x:v>439339</x:v>
       </x:c>
-      <x:c r="I18" s="8" t="n">
+      <x:c r="I18" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J18" s="10" t="n">
+      <x:c r="J18" s="48" t="n">
         <x:v>61.2</x:v>
       </x:c>
-      <x:c r="K18" s="10" t="n">
+      <x:c r="K18" s="48" t="n">
         <x:v>2.3</x:v>
       </x:c>
-      <x:c r="L18" s="7" t="str">
+      <x:c r="L18" s="45" t="str">
         <x:v>对照</x:v>
       </x:c>
-      <x:c r="M18" s="7" t="str">
+      <x:c r="M18" s="49" t="str">
         <x:v>无</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="15" t="str">
+      <x:c r="A19" s="62" t="str">
         <x:v>tlfloat_quad_arithmetic</x:v>
       </x:c>
-      <x:c r="B19" s="15" t="str">
+      <x:c r="B19" s="63" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C19" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D19" s="16" t="n">
+      <x:c r="C19" s="63" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D19" s="64" t="n">
         <x:v>3.29</x:v>
       </x:c>
-      <x:c r="E19" s="16" t="n">
+      <x:c r="E19" s="64" t="n">
         <x:v>-2.77</x:v>
       </x:c>
-      <x:c r="F19" s="17" t="n">
+      <x:c r="F19" s="65" t="n">
         <x:v>39387014</x:v>
       </x:c>
-      <x:c r="G19" s="16" t="n">
+      <x:c r="G19" s="64" t="n">
         <x:v>86.93</x:v>
       </x:c>
-      <x:c r="H19" s="17" t="n">
+      <x:c r="H19" s="65" t="n">
         <x:v>516102</x:v>
       </x:c>
-      <x:c r="I19" s="16" t="n">
+      <x:c r="I19" s="64" t="n">
         <x:v>17.47</x:v>
       </x:c>
-      <x:c r="J19" s="18" t="n">
+      <x:c r="J19" s="66" t="n">
         <x:v>98.3</x:v>
       </x:c>
-      <x:c r="K19" s="18" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L19" s="15" t="str">
+      <x:c r="K19" s="66" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L19" s="63" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="M19" s="15" t="str">
+      <x:c r="M19" s="67" t="str">
         <x:v>无</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
-      <x:c r="A20" s="25" t="str">
+      <x:c r="A20" s="50" t="str">
         <x:v>tlfloat_quad_arithmetic</x:v>
       </x:c>
-      <x:c r="B20" s="25" t="str">
+      <x:c r="B20" s="51" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C20" s="25" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D20" s="26" t="n">
+      <x:c r="C20" s="51" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D20" s="52" t="n">
         <x:v>15.78</x:v>
       </x:c>
-      <x:c r="E20" s="26" t="n">
+      <x:c r="E20" s="52" t="n">
         <x:v>9.72</x:v>
       </x:c>
-      <x:c r="F20" s="27" t="n">
+      <x:c r="F20" s="53" t="n">
         <x:v>28139344</x:v>
       </x:c>
-      <x:c r="G20" s="26" t="n">
+      <x:c r="G20" s="52" t="n">
         <x:v>33.55</x:v>
       </x:c>
-      <x:c r="H20" s="27" t="n">
+      <x:c r="H20" s="53" t="n">
         <x:v>487120</x:v>
       </x:c>
-      <x:c r="I20" s="26" t="n">
+      <x:c r="I20" s="52" t="n">
         <x:v>10.88</x:v>
       </x:c>
-      <x:c r="J20" s="28" t="n">
+      <x:c r="J20" s="54" t="n">
         <x:v>80.2</x:v>
       </x:c>
-      <x:c r="K20" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L20" s="25" t="str">
+      <x:c r="K20" s="54" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L20" s="51" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M20" s="25" t="str">
+      <x:c r="M20" s="55" t="str">
         <x:v>性能</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
-      <x:c r="A21" s="25" t="str">
+      <x:c r="A21" s="56" t="str">
         <x:v>tlfloat_quad_arithmetic</x:v>
       </x:c>
-      <x:c r="B21" s="25" t="str">
+      <x:c r="B21" s="57" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="C21" s="25" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D21" s="26" t="n">
+      <x:c r="C21" s="57" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D21" s="58" t="n">
         <x:v>3.67</x:v>
       </x:c>
-      <x:c r="E21" s="26" t="n">
+      <x:c r="E21" s="58" t="n">
         <x:v>-2.39</x:v>
       </x:c>
-      <x:c r="F21" s="27" t="n">
+      <x:c r="F21" s="59" t="n">
         <x:v>35644212</x:v>
       </x:c>
-      <x:c r="G21" s="26" t="n">
+      <x:c r="G21" s="58" t="n">
         <x:v>69.17</x:v>
       </x:c>
-      <x:c r="H21" s="27" t="n">
+      <x:c r="H21" s="59" t="n">
         <x:v>430132</x:v>
       </x:c>
-      <x:c r="I21" s="26" t="n">
+      <x:c r="I21" s="58" t="n">
         <x:v>-2.1</x:v>
       </x:c>
-      <x:c r="J21" s="28" t="n">
+      <x:c r="J21" s="60" t="n">
         <x:v>89.8</x:v>
       </x:c>
-      <x:c r="K21" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L21" s="25" t="str">
+      <x:c r="K21" s="60" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L21" s="57" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="M21" s="25" t="str">
+      <x:c r="M21" s="61" t="str">
         <x:v>非缓存Token</x:v>
       </x:c>
     </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="38"/>
+      <x:c r="B22" s="38"/>
+      <x:c r="C22" s="38"/>
+      <x:c r="D22" s="38"/>
+      <x:c r="E22" s="38"/>
+      <x:c r="F22" s="38"/>
+      <x:c r="G22" s="38"/>
+      <x:c r="H22" s="38"/>
+      <x:c r="I22" s="38"/>
+      <x:c r="J22" s="38"/>
+      <x:c r="K22" s="38"/>
+      <x:c r="L22" s="38"/>
+      <x:c r="M22" s="38"/>
+    </x:row>
     <x:row r="23">
-      <x:c r="A23" s="20" t="str">
+      <x:c r="A23" s="39" t="str">
         <x:v>口径</x:v>
       </x:c>
-      <x:c r="B23" s="20" t="str">
+      <x:c r="B23" s="39" t="str">
         <x:v>同一算子四组共有重复轮次</x:v>
       </x:c>
-      <x:c r="C23" s="20" t="str">
+      <x:c r="C23" s="39" t="str">
         <x:v>GF仅1–2轮；其余1–3轮</x:v>
       </x:c>
-      <x:c r="D23" s="20" t="str">
+      <x:c r="D23" s="39" t="str">
         <x:v>得分为本轮相对自身基线的性能提升中位数</x:v>
       </x:c>
-      <x:c r="E23" s="20" t="str">
+      <x:c r="E23" s="39" t="str">
         <x:v>diff=本组得分−A组得分（百分点）</x:v>
       </x:c>
-      <x:c r="F23" s="20" t="str">
+      <x:c r="F23" s="39" t="str">
         <x:v>总Token=非缓存Token+缓存读取Token</x:v>
       </x:c>
-      <x:c r="G23" s="20" t="str">
+      <x:c r="G23" s="39" t="str">
         <x:v>负值表示较A节省</x:v>
       </x:c>
-      <x:c r="H23" s="20" t="str">
+      <x:c r="H23" s="39" t="str">
         <x:v>非缓存Token不含缓存读取</x:v>
       </x:c>
-      <x:c r="I23" s="20" t="str">
+      <x:c r="I23" s="39" t="str">
         <x:v>负值表示较A节省</x:v>
       </x:c>
-      <x:c r="J23" s="20" t="str">
+      <x:c r="J23" s="39" t="str">
         <x:v>墙钟时间中位数</x:v>
       </x:c>
-      <x:c r="K23" s="20" t="str">
+      <x:c r="K23" s="39" t="str">
         <x:v>轮数均值</x:v>
       </x:c>
-      <x:c r="L23" s="20" t="str">
+      <x:c r="L23" s="39" t="str">
         <x:v>性能提升或任一Token下降即“是”</x:v>
       </x:c>
-      <x:c r="M23" s="20" t="str">
+      <x:c r="M23" s="39" t="str">
         <x:v>优势依据列列出触发条件</x:v>
       </x:c>
     </x:row>
@@ -1264,87 +1390,87 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="23" t="str">
+      <x:c r="A1" s="43" t="str">
         <x:v>组别</x:v>
       </x:c>
-      <x:c r="B1" s="23" t="str">
+      <x:c r="B1" s="43" t="str">
         <x:v>OpenWiki使用</x:v>
       </x:c>
-      <x:c r="C1" s="23" t="str">
+      <x:c r="C1" s="43" t="str">
         <x:v>源码检索范围</x:v>
       </x:c>
-      <x:c r="D1" s="23" t="str">
+      <x:c r="D1" s="43" t="str">
         <x:v>执行规则</x:v>
       </x:c>
-      <x:c r="E1" s="23" t="str">
+      <x:c r="E1" s="43" t="str">
         <x:v>对照说明</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="24" t="str">
+      <x:c r="A2" s="41" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="B2" s="24" t="str">
+      <x:c r="B2" s="41" t="str">
         <x:v>不读取Wiki</x:v>
       </x:c>
-      <x:c r="C2" s="24" t="str">
+      <x:c r="C2" s="41" t="str">
         <x:v>原始源码搜索</x:v>
       </x:c>
-      <x:c r="D2" s="24" t="str">
+      <x:c r="D2" s="41" t="str">
         <x:v>原始optimizer流程</x:v>
       </x:c>
-      <x:c r="E2" s="24" t="str">
+      <x:c r="E2" s="41" t="str">
         <x:v>每个算子单独以A为baseline</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="24" t="str">
+      <x:c r="A3" s="41" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="B3" s="24" t="str">
+      <x:c r="B3" s="41" t="str">
         <x:v>搜索阶段参考Wiki</x:v>
       </x:c>
-      <x:c r="C3" s="24" t="str">
+      <x:c r="C3" s="41" t="str">
         <x:v>源码grep不设额外范围限制</x:v>
       </x:c>
-      <x:c r="D3" s="24" t="str">
+      <x:c r="D3" s="41" t="str">
         <x:v>其余沿用原流程</x:v>
       </x:c>
-      <x:c r="E3" s="24" t="str">
+      <x:c r="E3" s="41" t="str">
         <x:v>检验增加Wiki参考的影响</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
-      <x:c r="A4" s="24" t="str">
+      <x:c r="A4" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="B4" s="24" t="str">
+      <x:c r="B4" s="41" t="str">
         <x:v>Wiki导航后定向搜索</x:v>
       </x:c>
-      <x:c r="C4" s="24" t="str">
+      <x:c r="C4" s="41" t="str">
         <x:v>首轮最多5文件/2目录；未命中扩展一次</x:v>
       </x:c>
-      <x:c r="D4" s="24" t="str">
+      <x:c r="D4" s="41" t="str">
         <x:v>按Wiki引导缩小搜索范围</x:v>
       </x:c>
-      <x:c r="E4" s="24" t="str">
+      <x:c r="E4" s="41" t="str">
         <x:v>检验受限定向搜索的影响</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="24" t="str">
+      <x:c r="A5" s="41" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="B5" s="24" t="str">
+      <x:c r="B5" s="41" t="str">
         <x:v>按触发规则读取Wiki</x:v>
       </x:c>
-      <x:c r="C5" s="24" t="str">
+      <x:c r="C5" s="41" t="str">
         <x:v>禁止无边界全仓搜索</x:v>
       </x:c>
-      <x:c r="D5" s="24" t="str">
+      <x:c r="D5" s="41" t="str">
         <x:v>原optimizer skill+根AGENTS.md；改架构前读index.md，构建/测试前读quickstart.md</x:v>
       </x:c>
-      <x:c r="E5" s="24" t="str">
+      <x:c r="E5" s="41" t="str">
         <x:v>检验强制阅读规则的影响</x:v>
       </x:c>
     </x:row>
@@ -1362,66 +1488,66 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="23" t="str">
+      <x:c r="A1" s="43" t="str">
         <x:v>项目</x:v>
       </x:c>
-      <x:c r="B1" s="23" t="str">
+      <x:c r="B1" s="43" t="str">
         <x:v>说明</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
-      <x:c r="A2" s="24" t="str">
+      <x:c r="A2" s="41" t="str">
         <x:v>源明细</x:v>
       </x:c>
-      <x:c r="B2" s="24" t="str">
+      <x:c r="B2" s="41" t="str">
         <x:v>session-results-2026-09-28.tsv；仅纳入formal且状态为正式有效的行</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="38" customHeight="1">
-      <x:c r="A3" s="24" t="str">
+      <x:c r="A3" s="41" t="str">
         <x:v>可比样本</x:v>
       </x:c>
-      <x:c r="B3" s="24" t="str">
+      <x:c r="B3" s="41" t="str">
         <x:v>每个算子仅保留A/B/C/D四组均有效的重复轮次；GF C3缺失，故GF只用前两轮</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="24" t="str">
+      <x:c r="A4" s="41" t="str">
         <x:v>性能得分</x:v>
       </x:c>
-      <x:c r="B4" s="24" t="str">
+      <x:c r="B4" s="41" t="str">
         <x:v>每条session相对其自身baseline的性能提升百分比；组得分取可比轮次中位数；不是eval_framework官方分数</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
-      <x:c r="A5" s="24" t="str">
+      <x:c r="A5" s="41" t="str">
         <x:v>diff</x:v>
       </x:c>
-      <x:c r="B5" s="24" t="str">
+      <x:c r="B5" s="41" t="str">
         <x:v>本组性能得分减同算子A组性能得分，单位为百分点；正值表示提升</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
-      <x:c r="A6" s="24" t="str">
+      <x:c r="A6" s="41" t="str">
         <x:v>Token</x:v>
       </x:c>
-      <x:c r="B6" s="24" t="str">
+      <x:c r="B6" s="41" t="str">
         <x:v>总Token按每条session的非缓存Token+缓存读取Token计算，再取组中位数；非缓存Token另取组中位数</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
-      <x:c r="A7" s="24" t="str">
+      <x:c r="A7" s="41" t="str">
         <x:v>优势组</x:v>
       </x:c>
-      <x:c r="B7" s="24" t="str">
+      <x:c r="B7" s="41" t="str">
         <x:v>仅B/C/D判断：性能得分高于A，或总Token中位数低于A，或非缓存Token中位数低于A。任一成立即是；耗时不参与判定</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
-      <x:c r="A8" s="24" t="str">
+      <x:c r="A8" s="41" t="str">
         <x:v>限制</x:v>
       </x:c>
-      <x:c r="B8" s="24" t="str">
+      <x:c r="B8" s="41" t="str">
         <x:v>这是原优化session结果，尚未完成统一低负载复测；OpenWiki生成成本未计入各session Token；不宣称因果显著性</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add mean variance and A-control comparisons to optimizer results
</commit_message>
<xml_diff>
--- a/experiments/openwiki-optimizer-920c-2026-09/a-baseline-advantage-2026-09-28.xlsx
+++ b/experiments/openwiki-optimizer-920c-2026-09/a-baseline-advantage-2026-09-28.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A组对照" sheetId="1" r:id="Ra78bed7b4ae24083"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="组别区别" sheetId="2" r:id="R2619c228e24f459e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与限制" sheetId="3" r:id="R6b63534008bc4d1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A组对照" sheetId="1" r:id="Re343e5e000014d04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="组别区别" sheetId="2" r:id="R63d1583db84049a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与限制" sheetId="3" r:id="R854acc28c43145a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,12 +15,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="0.00"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0.0"/>
+    <x:numFmt numFmtId="203" formatCode="0.0000"/>
+    <x:numFmt numFmtId="204" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="205" formatCode="0.000E+00"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -68,6 +71,18 @@
       <x:color rgb="FF222222"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF274C72"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
   <x:fills count="7">
     <x:fill>
@@ -102,7 +117,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="9">
+  <x:borders count="14">
     <x:border/>
     <x:border>
       <x:left style="thick">
@@ -156,11 +171,42 @@
         <x:color rgb="FF333333"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:top style="medium">
+        <x:color rgb="FF333333"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="medium">
+        <x:color rgb="FF333333"/>
+      </x:right>
+      <x:top style="medium">
+        <x:color rgb="FF333333"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="medium">
+        <x:color rgb="FF333333"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:bottom style="medium">
+        <x:color rgb="FF333333"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="medium">
+        <x:color rgb="FF333333"/>
+      </x:right>
+      <x:bottom style="medium">
+        <x:color rgb="FF333333"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="74">
+  <x:cellXfs count="101">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -239,6 +285,87 @@
     <x:xf numFmtId="201" fontId="1" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="1" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="10" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="10" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="10" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -454,9 +581,18 @@
     <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="11" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="32" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="21" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="25" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="29" customHeight="1">
+    <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="42" t="str">
         <x:v>算子</x:v>
       </x:c>
@@ -495,6 +631,33 @@
       </x:c>
       <x:c r="M1" s="42" t="str">
         <x:v>优势依据</x:v>
+      </x:c>
+      <x:c r="N1" s="80" t="str">
+        <x:v>性能均值(%)</x:v>
+      </x:c>
+      <x:c r="O1" s="80" t="str">
+        <x:v>性能样本方差(pp²)</x:v>
+      </x:c>
+      <x:c r="P1" s="80" t="str">
+        <x:v>性能均值diff(pp)</x:v>
+      </x:c>
+      <x:c r="Q1" s="80" t="str">
+        <x:v>总Token均值</x:v>
+      </x:c>
+      <x:c r="R1" s="80" t="str">
+        <x:v>总Token样本方差(Token²)</x:v>
+      </x:c>
+      <x:c r="S1" s="80" t="str">
+        <x:v>总Token均值较A(%)</x:v>
+      </x:c>
+      <x:c r="T1" s="80" t="str">
+        <x:v>非缓存Token均值</x:v>
+      </x:c>
+      <x:c r="U1" s="80" t="str">
+        <x:v>非缓存Token样本方差(Token²)</x:v>
+      </x:c>
+      <x:c r="V1" s="80" t="str">
+        <x:v>非缓存Token均值较A(%)</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
@@ -537,6 +700,33 @@
       <x:c r="M2" s="49" t="str">
         <x:v>无</x:v>
       </x:c>
+      <x:c r="N2" s="81" t="n">
+        <x:v>20.49525</x:v>
+      </x:c>
+      <x:c r="O2" s="81" t="n">
+        <x:v>0.00041760500000000427</x:v>
+      </x:c>
+      <x:c r="P2" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q2" s="82" t="n">
+        <x:v>24589065</x:v>
+      </x:c>
+      <x:c r="R2" s="83" t="n">
+        <x:v>222592846565888</x:v>
+      </x:c>
+      <x:c r="S2" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T2" s="82" t="n">
+        <x:v>437865</x:v>
+      </x:c>
+      <x:c r="U2" s="83" t="n">
+        <x:v>3005915648</x:v>
+      </x:c>
+      <x:c r="V2" s="84" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="50" t="str">
@@ -578,6 +768,33 @@
       <x:c r="M3" s="55" t="str">
         <x:v>性能；总Token；非缓存Token</x:v>
       </x:c>
+      <x:c r="N3" s="93" t="n">
+        <x:v>26.78355</x:v>
+      </x:c>
+      <x:c r="O3" s="93" t="n">
+        <x:v>107.03746984500005</x:v>
+      </x:c>
+      <x:c r="P3" s="93" t="n">
+        <x:v>6.288300000000003</x:v>
+      </x:c>
+      <x:c r="Q3" s="94" t="n">
+        <x:v>11652755</x:v>
+      </x:c>
+      <x:c r="R3" s="95" t="n">
+        <x:v>38289265419528</x:v>
+      </x:c>
+      <x:c r="S3" s="93" t="n">
+        <x:v>-52.61001180809437</x:v>
+      </x:c>
+      <x:c r="T3" s="94" t="n">
+        <x:v>312851</x:v>
+      </x:c>
+      <x:c r="U3" s="95" t="n">
+        <x:v>9976063752</x:v>
+      </x:c>
+      <x:c r="V3" s="96" t="n">
+        <x:v>-28.550809039315773</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="50" t="str">
@@ -619,6 +836,33 @@
       <x:c r="M4" s="55" t="str">
         <x:v>总Token；非缓存Token</x:v>
       </x:c>
+      <x:c r="N4" s="93" t="n">
+        <x:v>18.3094</x:v>
+      </x:c>
+      <x:c r="O4" s="93" t="n">
+        <x:v>0.002888000000000039</x:v>
+      </x:c>
+      <x:c r="P4" s="93" t="n">
+        <x:v>-2.1858499999999985</x:v>
+      </x:c>
+      <x:c r="Q4" s="94" t="n">
+        <x:v>9608260.5</x:v>
+      </x:c>
+      <x:c r="R4" s="95" t="n">
+        <x:v>4940704963920.5</x:v>
+      </x:c>
+      <x:c r="S4" s="93" t="n">
+        <x:v>-60.92466102310112</x:v>
+      </x:c>
+      <x:c r="T4" s="94" t="n">
+        <x:v>273604.5</x:v>
+      </x:c>
+      <x:c r="U4" s="95" t="n">
+        <x:v>71413200.5</x:v>
+      </x:c>
+      <x:c r="V4" s="96" t="n">
+        <x:v>-37.51395978212463</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="56" t="str">
@@ -660,6 +904,33 @@
       <x:c r="M5" s="61" t="str">
         <x:v>性能；总Token</x:v>
       </x:c>
+      <x:c r="N5" s="97" t="n">
+        <x:v>26.27825</x:v>
+      </x:c>
+      <x:c r="O5" s="97" t="n">
+        <x:v>68.35260120499996</x:v>
+      </x:c>
+      <x:c r="P5" s="97" t="n">
+        <x:v>5.783000000000001</x:v>
+      </x:c>
+      <x:c r="Q5" s="98" t="n">
+        <x:v>13291914.5</x:v>
+      </x:c>
+      <x:c r="R5" s="99" t="n">
+        <x:v>20510853211380.5</x:v>
+      </x:c>
+      <x:c r="S5" s="97" t="n">
+        <x:v>-45.943798595025875</x:v>
+      </x:c>
+      <x:c r="T5" s="98" t="n">
+        <x:v>444714.5</x:v>
+      </x:c>
+      <x:c r="U5" s="99" t="n">
+        <x:v>67154894644.5</x:v>
+      </x:c>
+      <x:c r="V5" s="100" t="n">
+        <x:v>1.5642949310860743</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="44" t="str">
@@ -701,6 +972,33 @@
       <x:c r="M6" s="49" t="str">
         <x:v>无</x:v>
       </x:c>
+      <x:c r="N6" s="81" t="n">
+        <x:v>35.03273333333333</x:v>
+      </x:c>
+      <x:c r="O6" s="81" t="n">
+        <x:v>556.3578199433333</x:v>
+      </x:c>
+      <x:c r="P6" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q6" s="82" t="n">
+        <x:v>62907495</x:v>
+      </x:c>
+      <x:c r="R6" s="83" t="n">
+        <x:v>593135761792732</x:v>
+      </x:c>
+      <x:c r="S6" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T6" s="82" t="n">
+        <x:v>688508.3333333334</x:v>
+      </x:c>
+      <x:c r="U6" s="83" t="n">
+        <x:v>12266730801.333334</x:v>
+      </x:c>
+      <x:c r="V6" s="84" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="50" t="str">
@@ -742,6 +1040,33 @@
       <x:c r="M7" s="55" t="str">
         <x:v>性能；总Token</x:v>
       </x:c>
+      <x:c r="N7" s="93" t="n">
+        <x:v>46.2485</x:v>
+      </x:c>
+      <x:c r="O7" s="93" t="n">
+        <x:v>136.68181059</x:v>
+      </x:c>
+      <x:c r="P7" s="93" t="n">
+        <x:v>11.215766666666667</x:v>
+      </x:c>
+      <x:c r="Q7" s="94" t="n">
+        <x:v>64878170</x:v>
+      </x:c>
+      <x:c r="R7" s="95" t="n">
+        <x:v>376453457651100</x:v>
+      </x:c>
+      <x:c r="S7" s="93" t="n">
+        <x:v>3.1326553378099087</x:v>
+      </x:c>
+      <x:c r="T7" s="94" t="n">
+        <x:v>874543.3333333334</x:v>
+      </x:c>
+      <x:c r="U7" s="95" t="n">
+        <x:v>11318193521.333334</x:v>
+      </x:c>
+      <x:c r="V7" s="96" t="n">
+        <x:v>27.02000702000702</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="50" t="str">
@@ -783,6 +1108,33 @@
       <x:c r="M8" s="55" t="str">
         <x:v>总Token</x:v>
       </x:c>
+      <x:c r="N8" s="93" t="n">
+        <x:v>28.760166666666667</x:v>
+      </x:c>
+      <x:c r="O8" s="93" t="n">
+        <x:v>827.9729256633334</x:v>
+      </x:c>
+      <x:c r="P8" s="93" t="n">
+        <x:v>-6.272566666666666</x:v>
+      </x:c>
+      <x:c r="Q8" s="94" t="n">
+        <x:v>50066340.333333336</x:v>
+      </x:c>
+      <x:c r="R8" s="95" t="n">
+        <x:v>480361589557258.3</x:v>
+      </x:c>
+      <x:c r="S8" s="93" t="n">
+        <x:v>-20.41275791806153</x:v>
+      </x:c>
+      <x:c r="T8" s="94" t="n">
+        <x:v>737828.3333333334</x:v>
+      </x:c>
+      <x:c r="U8" s="95" t="n">
+        <x:v>50920443786.33333</x:v>
+      </x:c>
+      <x:c r="V8" s="96" t="n">
+        <x:v>7.163311990898191</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="56" t="str">
@@ -824,6 +1176,33 @@
       <x:c r="M9" s="61" t="str">
         <x:v>性能；总Token；非缓存Token</x:v>
       </x:c>
+      <x:c r="N9" s="97" t="n">
+        <x:v>37.68156666666667</x:v>
+      </x:c>
+      <x:c r="O9" s="97" t="n">
+        <x:v>233.34182512333334</x:v>
+      </x:c>
+      <x:c r="P9" s="97" t="n">
+        <x:v>2.648833333333336</x:v>
+      </x:c>
+      <x:c r="Q9" s="98" t="n">
+        <x:v>43890639</x:v>
+      </x:c>
+      <x:c r="R9" s="99" t="n">
+        <x:v>752033194500333</x:v>
+      </x:c>
+      <x:c r="S9" s="97" t="n">
+        <x:v>-30.22987324483355</x:v>
+      </x:c>
+      <x:c r="T9" s="98" t="n">
+        <x:v>598543</x:v>
+      </x:c>
+      <x:c r="U9" s="99" t="n">
+        <x:v>33222381997</x:v>
+      </x:c>
+      <x:c r="V9" s="100" t="n">
+        <x:v>-13.066702170150446</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="44" t="str">
@@ -865,6 +1244,33 @@
       <x:c r="M10" s="49" t="str">
         <x:v>无</x:v>
       </x:c>
+      <x:c r="N10" s="81" t="n">
+        <x:v>8.149133333333332</x:v>
+      </x:c>
+      <x:c r="O10" s="81" t="n">
+        <x:v>0.22454137333333307</x:v>
+      </x:c>
+      <x:c r="P10" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q10" s="82" t="n">
+        <x:v>22963242</x:v>
+      </x:c>
+      <x:c r="R10" s="83" t="n">
+        <x:v>37169134555651</x:v>
+      </x:c>
+      <x:c r="S10" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T10" s="82" t="n">
+        <x:v>486143.3333333333</x:v>
+      </x:c>
+      <x:c r="U10" s="83" t="n">
+        <x:v>30259032792.333332</x:v>
+      </x:c>
+      <x:c r="V10" s="84" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="50" t="str">
@@ -906,6 +1312,33 @@
       <x:c r="M11" s="55" t="str">
         <x:v>非缓存Token</x:v>
       </x:c>
+      <x:c r="N11" s="93" t="n">
+        <x:v>3.5949000000000004</x:v>
+      </x:c>
+      <x:c r="O11" s="93" t="n">
+        <x:v>2.58580525</x:v>
+      </x:c>
+      <x:c r="P11" s="93" t="n">
+        <x:v>-4.554233333333331</x:v>
+      </x:c>
+      <x:c r="Q11" s="94" t="n">
+        <x:v>25589182.666666668</x:v>
+      </x:c>
+      <x:c r="R11" s="95" t="n">
+        <x:v>18951539469484.332</x:v>
+      </x:c>
+      <x:c r="S11" s="93" t="n">
+        <x:v>11.43540910585128</x:v>
+      </x:c>
+      <x:c r="T11" s="94" t="n">
+        <x:v>413652</x:v>
+      </x:c>
+      <x:c r="U11" s="95" t="n">
+        <x:v>858857239</x:v>
+      </x:c>
+      <x:c r="V11" s="96" t="n">
+        <x:v>-14.911514436757333</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="62" t="str">
@@ -947,6 +1380,33 @@
       <x:c r="M12" s="67" t="str">
         <x:v>无</x:v>
       </x:c>
+      <x:c r="N12" s="85" t="n">
+        <x:v>4.560133333333333</x:v>
+      </x:c>
+      <x:c r="O12" s="85" t="n">
+        <x:v>3.045400663333333</x:v>
+      </x:c>
+      <x:c r="P12" s="85" t="n">
+        <x:v>-3.5889999999999986</x:v>
+      </x:c>
+      <x:c r="Q12" s="86" t="n">
+        <x:v>26825900</x:v>
+      </x:c>
+      <x:c r="R12" s="87" t="n">
+        <x:v>80846224213159</x:v>
+      </x:c>
+      <x:c r="S12" s="85" t="n">
+        <x:v>16.821048177779076</x:v>
+      </x:c>
+      <x:c r="T12" s="86" t="n">
+        <x:v>434113.3333333333</x:v>
+      </x:c>
+      <x:c r="U12" s="87" t="n">
+        <x:v>1243074108.3333333</x:v>
+      </x:c>
+      <x:c r="V12" s="88" t="n">
+        <x:v>-10.702604855906694</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="68" t="str">
@@ -988,6 +1448,33 @@
       <x:c r="M13" s="73" t="str">
         <x:v>无</x:v>
       </x:c>
+      <x:c r="N13" s="89" t="n">
+        <x:v>4.272966666666666</x:v>
+      </x:c>
+      <x:c r="O13" s="89" t="n">
+        <x:v>27.913579293333328</x:v>
+      </x:c>
+      <x:c r="P13" s="89" t="n">
+        <x:v>-3.8761666666666654</x:v>
+      </x:c>
+      <x:c r="Q13" s="90" t="n">
+        <x:v>35963106</x:v>
+      </x:c>
+      <x:c r="R13" s="91" t="n">
+        <x:v>65376592927344</x:v>
+      </x:c>
+      <x:c r="S13" s="89" t="n">
+        <x:v>56.61162304521288</x:v>
+      </x:c>
+      <x:c r="T13" s="90" t="n">
+        <x:v>545314</x:v>
+      </x:c>
+      <x:c r="U13" s="91" t="n">
+        <x:v>29331240304</x:v>
+      </x:c>
+      <x:c r="V13" s="92" t="n">
+        <x:v>12.17144463566986</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="44" t="str">
@@ -1029,6 +1516,33 @@
       <x:c r="M14" s="49" t="str">
         <x:v>无</x:v>
       </x:c>
+      <x:c r="N14" s="81" t="n">
+        <x:v>21.580466666666666</x:v>
+      </x:c>
+      <x:c r="O14" s="81" t="n">
+        <x:v>87.10974770333334</x:v>
+      </x:c>
+      <x:c r="P14" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q14" s="82" t="n">
+        <x:v>56144683</x:v>
+      </x:c>
+      <x:c r="R14" s="83" t="n">
+        <x:v>1011085820256433</x:v>
+      </x:c>
+      <x:c r="S14" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T14" s="82" t="n">
+        <x:v>587883</x:v>
+      </x:c>
+      <x:c r="U14" s="83" t="n">
+        <x:v>92305084017</x:v>
+      </x:c>
+      <x:c r="V14" s="84" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="50" t="str">
@@ -1070,6 +1584,33 @@
       <x:c r="M15" s="55" t="str">
         <x:v>总Token；非缓存Token</x:v>
       </x:c>
+      <x:c r="N15" s="93" t="n">
+        <x:v>21.600666666666665</x:v>
+      </x:c>
+      <x:c r="O15" s="93" t="n">
+        <x:v>7.920882643333333</x:v>
+      </x:c>
+      <x:c r="P15" s="93" t="n">
+        <x:v>0.020199999999999108</x:v>
+      </x:c>
+      <x:c r="Q15" s="94" t="n">
+        <x:v>30122942</x:v>
+      </x:c>
+      <x:c r="R15" s="95" t="n">
+        <x:v>25391573808841</x:v>
+      </x:c>
+      <x:c r="S15" s="93" t="n">
+        <x:v>-46.34764969641025</x:v>
+      </x:c>
+      <x:c r="T15" s="94" t="n">
+        <x:v>572371.3333333334</x:v>
+      </x:c>
+      <x:c r="U15" s="95" t="n">
+        <x:v>61514861406.33333</x:v>
+      </x:c>
+      <x:c r="V15" s="96" t="n">
+        <x:v>-2.6385635690548304</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="50" t="str">
@@ -1111,6 +1652,33 @@
       <x:c r="M16" s="55" t="str">
         <x:v>性能；总Token；非缓存Token</x:v>
       </x:c>
+      <x:c r="N16" s="93" t="n">
+        <x:v>21.973399999999998</x:v>
+      </x:c>
+      <x:c r="O16" s="93" t="n">
+        <x:v>13.691935559999992</x:v>
+      </x:c>
+      <x:c r="P16" s="93" t="n">
+        <x:v>0.3929333333333318</x:v>
+      </x:c>
+      <x:c r="Q16" s="94" t="n">
+        <x:v>36613946</x:v>
+      </x:c>
+      <x:c r="R16" s="95" t="n">
+        <x:v>272252489556451</x:v>
+      </x:c>
+      <x:c r="S16" s="93" t="n">
+        <x:v>-34.78644095292158</x:v>
+      </x:c>
+      <x:c r="T16" s="94" t="n">
+        <x:v>510820.6666666667</x:v>
+      </x:c>
+      <x:c r="U16" s="95" t="n">
+        <x:v>42204637752.33333</x:v>
+      </x:c>
+      <x:c r="V16" s="96" t="n">
+        <x:v>-13.10844731576407</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="56" t="str">
@@ -1152,6 +1720,33 @@
       <x:c r="M17" s="61" t="str">
         <x:v>性能；总Token</x:v>
       </x:c>
+      <x:c r="N17" s="97" t="n">
+        <x:v>25.686700000000002</x:v>
+      </x:c>
+      <x:c r="O17" s="97" t="n">
+        <x:v>122.72971515999998</x:v>
+      </x:c>
+      <x:c r="P17" s="97" t="n">
+        <x:v>4.106233333333336</x:v>
+      </x:c>
+      <x:c r="Q17" s="98" t="n">
+        <x:v>35683880</x:v>
+      </x:c>
+      <x:c r="R17" s="99" t="n">
+        <x:v>271666743027573</x:v>
+      </x:c>
+      <x:c r="S17" s="97" t="n">
+        <x:v>-36.44299318601549</x:v>
+      </x:c>
+      <x:c r="T17" s="98" t="n">
+        <x:v>674962.6666666666</x:v>
+      </x:c>
+      <x:c r="U17" s="99" t="n">
+        <x:v>87471672266.33333</x:v>
+      </x:c>
+      <x:c r="V17" s="100" t="n">
+        <x:v>14.812414488370408</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="44" t="str">
@@ -1193,6 +1788,33 @@
       <x:c r="M18" s="49" t="str">
         <x:v>无</x:v>
       </x:c>
+      <x:c r="N18" s="81" t="n">
+        <x:v>5.525566666666666</x:v>
+      </x:c>
+      <x:c r="O18" s="81" t="n">
+        <x:v>6.5809185433333335</x:v>
+      </x:c>
+      <x:c r="P18" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q18" s="82" t="n">
+        <x:v>23925296.666666668</x:v>
+      </x:c>
+      <x:c r="R18" s="83" t="n">
+        <x:v>152892348036654.3</x:v>
+      </x:c>
+      <x:c r="S18" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T18" s="82" t="n">
+        <x:v>541147.3333333334</x:v>
+      </x:c>
+      <x:c r="U18" s="83" t="n">
+        <x:v>45321871854.33333</x:v>
+      </x:c>
+      <x:c r="V18" s="84" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="62" t="str">
@@ -1234,6 +1856,33 @@
       <x:c r="M19" s="67" t="str">
         <x:v>无</x:v>
       </x:c>
+      <x:c r="N19" s="85" t="n">
+        <x:v>4.091266666666667</x:v>
+      </x:c>
+      <x:c r="O19" s="85" t="n">
+        <x:v>2.050432603333333</x:v>
+      </x:c>
+      <x:c r="P19" s="85" t="n">
+        <x:v>-1.4342999999999995</x:v>
+      </x:c>
+      <x:c r="Q19" s="86" t="n">
+        <x:v>38381270.333333336</x:v>
+      </x:c>
+      <x:c r="R19" s="87" t="n">
+        <x:v>256409207565132.3</x:v>
+      </x:c>
+      <x:c r="S19" s="85" t="n">
+        <x:v>60.42129327828607</x:v>
+      </x:c>
+      <x:c r="T19" s="86" t="n">
+        <x:v>572267.6666666666</x:v>
+      </x:c>
+      <x:c r="U19" s="87" t="n">
+        <x:v>29142840716.333336</x:v>
+      </x:c>
+      <x:c r="V19" s="88" t="n">
+        <x:v>5.7508060035406094</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="50" t="str">
@@ -1275,6 +1924,33 @@
       <x:c r="M20" s="55" t="str">
         <x:v>性能</x:v>
       </x:c>
+      <x:c r="N20" s="93" t="n">
+        <x:v>14.263833333333332</x:v>
+      </x:c>
+      <x:c r="O20" s="93" t="n">
+        <x:v>89.31588792333332</x:v>
+      </x:c>
+      <x:c r="P20" s="93" t="n">
+        <x:v>8.738266666666666</x:v>
+      </x:c>
+      <x:c r="Q20" s="94" t="n">
+        <x:v>31963363.333333332</x:v>
+      </x:c>
+      <x:c r="R20" s="95" t="n">
+        <x:v>63188127592305.34</x:v>
+      </x:c>
+      <x:c r="S20" s="93" t="n">
+        <x:v>33.59651827375458</x:v>
+      </x:c>
+      <x:c r="T20" s="94" t="n">
+        <x:v>527011.3333333334</x:v>
+      </x:c>
+      <x:c r="U20" s="95" t="n">
+        <x:v>5597536625.333334</x:v>
+      </x:c>
+      <x:c r="V20" s="96" t="n">
+        <x:v>-2.612227600370076</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="56" t="str">
@@ -1315,6 +1991,33 @@
       </x:c>
       <x:c r="M21" s="61" t="str">
         <x:v>非缓存Token</x:v>
+      </x:c>
+      <x:c r="N21" s="97" t="n">
+        <x:v>7.914533333333334</x:v>
+      </x:c>
+      <x:c r="O21" s="97" t="n">
+        <x:v>57.214602303333336</x:v>
+      </x:c>
+      <x:c r="P21" s="97" t="n">
+        <x:v>2.3889666666666676</x:v>
+      </x:c>
+      <x:c r="Q21" s="98" t="n">
+        <x:v>36784407.666666664</x:v>
+      </x:c>
+      <x:c r="R21" s="99" t="n">
+        <x:v>383896510874734.4</x:v>
+      </x:c>
+      <x:c r="S21" s="97" t="n">
+        <x:v>53.74692393225635</x:v>
+      </x:c>
+      <x:c r="T21" s="98" t="n">
+        <x:v>480279.6666666667</x:v>
+      </x:c>
+      <x:c r="U21" s="99" t="n">
+        <x:v>28456232366.333336</x:v>
+      </x:c>
+      <x:c r="V21" s="100" t="n">
+        <x:v>-11.247891824900435</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1331,6 +2034,15 @@
       <x:c r="K22" s="38"/>
       <x:c r="L22" s="38"/>
       <x:c r="M22" s="38"/>
+      <x:c r="N22"/>
+      <x:c r="O22"/>
+      <x:c r="P22"/>
+      <x:c r="Q22"/>
+      <x:c r="R22"/>
+      <x:c r="S22"/>
+      <x:c r="T22"/>
+      <x:c r="U22"/>
+      <x:c r="V22"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="39" t="str">
@@ -1372,6 +2084,15 @@
       <x:c r="M23" s="39" t="str">
         <x:v>优势依据列列出触发条件</x:v>
       </x:c>
+      <x:c r="N23"/>
+      <x:c r="O23"/>
+      <x:c r="P23"/>
+      <x:c r="Q23"/>
+      <x:c r="R23"/>
+      <x:c r="S23"/>
+      <x:c r="T23"/>
+      <x:c r="U23"/>
+      <x:c r="V23"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1551,6 +2272,38 @@
         <x:v>这是原优化session结果，尚未完成统一低负载复测；OpenWiki生成成本未计入各session Token；不宣称因果显著性</x:v>
       </x:c>
     </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>统计样本</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>新增均值和方差仅用各算子四组共有的正式有效重复：GF为r1–r2，其他算子为r1–r3；GF其他组r3仍保留在逐次明细中。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>方差口径</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>性能提升、总Token、非缓存Token均使用样本方差（n−1）；性能方差单位为百分点平方，Token方差单位为Token平方。n仅2或3，方差描述波动，不构成显著性结论。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>均值与A比较</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>性能均值diff为本组均值减A组均值（百分点）；Token均值较A为本组均值/A组均值−1（百分比），负值表示节省。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>优势组标签</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>沿用原中位数规则，新增均值和方差不改变优势组判定。原实验性能未完成全算子统一低负载复测；不要将原session结果当作统一环境结论。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>